<commit_message>
feat: add Procfile Heroku configuration
</commit_message>
<xml_diff>
--- a/results/schedules/jadwal_piket_jt_express.xlsx
+++ b/results/schedules/jadwal_piket_jt_express.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J60"/>
+  <dimension ref="A1:J59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -619,9 +619,9 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
@@ -639,9 +639,9 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
+      <c r="J3" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
         </is>
       </c>
     </row>
@@ -661,9 +661,9 @@
           <t>Bebas</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
@@ -681,9 +681,9 @@
           <t>LIBUR</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
@@ -733,14 +733,14 @@
           <t>LIBUR</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="I5" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
@@ -765,14 +765,14 @@
           <t>Bebas</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
@@ -790,14 +790,14 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="I6" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="J6" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
         </is>
       </c>
     </row>
@@ -817,9 +817,9 @@
           <t>Bebas</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
@@ -842,9 +842,9 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="I7" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
@@ -869,9 +869,9 @@
           <t>Bebas</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
@@ -879,9 +879,9 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
@@ -889,14 +889,14 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="I8" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
@@ -921,9 +921,9 @@
           <t>Bebas</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
@@ -931,9 +931,9 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -941,9 +941,9 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="H9" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -951,9 +951,9 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="J9" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
         </is>
       </c>
     </row>
@@ -978,9 +978,9 @@
           <t>LIBUR</t>
         </is>
       </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
@@ -993,9 +993,9 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="H10" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
@@ -1040,9 +1040,9 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="G11" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
@@ -1055,9 +1055,9 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="J11" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
         </is>
       </c>
     </row>
@@ -1077,14 +1077,14 @@
           <t>Bebas</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
@@ -1092,14 +1092,14 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="G12" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="H12" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
@@ -1134,9 +1134,9 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
@@ -1144,19 +1144,19 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="H13" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="I13" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr">
@@ -1181,14 +1181,14 @@
           <t>Bebas</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
@@ -1196,9 +1196,9 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="G14" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
@@ -1211,9 +1211,9 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="J14" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
         </is>
       </c>
     </row>
@@ -1233,19 +1233,19 @@
           <t>Bebas</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="F15" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
@@ -1258,9 +1258,9 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="I15" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
@@ -1337,9 +1337,9 @@
           <t>Bebas</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
@@ -1347,19 +1347,19 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="F17" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="G17" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="H17" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
@@ -1394,9 +1394,9 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="E18" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
@@ -1404,9 +1404,9 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="G18" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
@@ -1414,14 +1414,14 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="I18" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="J18" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="J18" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
         </is>
       </c>
     </row>
@@ -1441,14 +1441,14 @@
           <t>Bebas</t>
         </is>
       </c>
-      <c r="D19" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="E19" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
@@ -1498,14 +1498,14 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="E20" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="F20" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
@@ -1513,14 +1513,14 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="H20" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="I20" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1550,9 +1550,9 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="E21" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
@@ -1565,9 +1565,9 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="H21" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
@@ -1602,9 +1602,9 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="E22" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
@@ -1617,19 +1617,19 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="H22" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="I22" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="J22" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="I22" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
         </is>
       </c>
     </row>
@@ -1649,14 +1649,14 @@
           <t>Bebas</t>
         </is>
       </c>
-      <c r="D23" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="E23" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
@@ -1669,14 +1669,14 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="H23" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="I23" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="I23" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -1701,14 +1701,14 @@
           <t>Bebas</t>
         </is>
       </c>
-      <c r="D24" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="E24" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
@@ -1753,14 +1753,14 @@
           <t>Bebas</t>
         </is>
       </c>
-      <c r="D25" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="E25" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
@@ -1773,9 +1773,9 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="H25" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
@@ -1783,9 +1783,9 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="J25" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
+      <c r="J25" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
         </is>
       </c>
     </row>
@@ -1867,19 +1867,19 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="F27" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="G27" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="H27" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="I27" s="4" t="inlineStr">
@@ -1887,9 +1887,9 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="J27" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
+      <c r="J27" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
         </is>
       </c>
     </row>
@@ -1909,9 +1909,9 @@
           <t>Bebas</t>
         </is>
       </c>
-      <c r="D28" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
@@ -1924,9 +1924,9 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="G28" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="H28" s="3" t="inlineStr">
@@ -1966,9 +1966,9 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="E29" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
@@ -1976,9 +1976,9 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="G29" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="H29" s="3" t="inlineStr">
@@ -2023,19 +2023,19 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="F30" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="G30" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="H30" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="H30" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="I30" s="4" t="inlineStr">
@@ -2043,9 +2043,9 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="J30" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
+      <c r="J30" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
         </is>
       </c>
     </row>
@@ -2070,9 +2070,9 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="E31" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
@@ -2085,9 +2085,9 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="H31" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
+      <c r="H31" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr">
@@ -2117,9 +2117,9 @@
           <t>Bebas</t>
         </is>
       </c>
-      <c r="D32" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
@@ -2132,14 +2132,14 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="G32" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="H32" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
+      <c r="G32" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="I32" s="4" t="inlineStr">
@@ -2147,9 +2147,9 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="J32" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
+      <c r="J32" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
         </is>
       </c>
     </row>
@@ -2169,14 +2169,14 @@
           <t>Bebas</t>
         </is>
       </c>
-      <c r="D33" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="E33" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
@@ -2184,14 +2184,14 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="G33" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="H33" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="H33" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="I33" s="4" t="inlineStr">
@@ -2221,9 +2221,9 @@
           <t>Bebas</t>
         </is>
       </c>
-      <c r="D34" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
@@ -2231,9 +2231,9 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="F34" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
@@ -2241,14 +2241,14 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="H34" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="I34" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="I34" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="J34" s="4" t="inlineStr">
@@ -2273,9 +2273,9 @@
           <t>Bebas</t>
         </is>
       </c>
-      <c r="D35" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr">
@@ -2303,9 +2303,9 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="J35" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
+      <c r="J35" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
         </is>
       </c>
     </row>
@@ -2325,9 +2325,9 @@
           <t>Bebas</t>
         </is>
       </c>
-      <c r="D36" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
@@ -2355,9 +2355,9 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="J36" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
+      <c r="J36" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
         </is>
       </c>
     </row>
@@ -2387,9 +2387,9 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="F37" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr">
@@ -2407,9 +2407,9 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="J37" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
+      <c r="J37" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
         </is>
       </c>
     </row>
@@ -2429,14 +2429,14 @@
           <t>Bebas</t>
         </is>
       </c>
-      <c r="D38" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="E38" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr">
@@ -2444,9 +2444,9 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="G38" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
+      <c r="G38" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr">
@@ -2459,9 +2459,9 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="J38" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
+      <c r="J38" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
         </is>
       </c>
     </row>
@@ -2481,24 +2481,24 @@
           <t>Bebas</t>
         </is>
       </c>
-      <c r="D39" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="E39" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="F39" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="G39" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr">
@@ -2538,24 +2538,24 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="E40" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="F40" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="G40" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="H40" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="G40" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="H40" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="I40" s="4" t="inlineStr">
@@ -2585,9 +2585,9 @@
           <t>Bebas</t>
         </is>
       </c>
-      <c r="D41" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
@@ -2595,9 +2595,9 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="F41" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="G41" s="4" t="inlineStr">
@@ -2610,14 +2610,14 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="I41" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="J41" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
+      <c r="I41" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="J41" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
         </is>
       </c>
     </row>
@@ -2642,9 +2642,9 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="E42" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
+      <c r="E42" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="F42" s="4" t="inlineStr">
@@ -2662,9 +2662,9 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="I42" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
+      <c r="I42" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="J42" s="3" t="inlineStr">
@@ -2709,9 +2709,9 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="H43" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
+      <c r="H43" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="I43" s="3" t="inlineStr">
@@ -2719,9 +2719,9 @@
           <t>LIBUR</t>
         </is>
       </c>
-      <c r="J43" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
+      <c r="J43" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
         </is>
       </c>
     </row>
@@ -2741,9 +2741,9 @@
           <t>JUMAT</t>
         </is>
       </c>
-      <c r="D44" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
@@ -2756,9 +2756,9 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="G44" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
+      <c r="G44" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="H44" s="3" t="inlineStr">
@@ -2793,14 +2793,14 @@
           <t>SABTU</t>
         </is>
       </c>
-      <c r="D45" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="E45" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
@@ -2845,9 +2845,9 @@
           <t>RABU</t>
         </is>
       </c>
-      <c r="D46" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
@@ -2870,9 +2870,9 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="I46" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
+      <c r="I46" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="J46" s="4" t="inlineStr">
@@ -2907,9 +2907,9 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="F47" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="G47" s="4" t="inlineStr">
@@ -2922,9 +2922,9 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="I47" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
+      <c r="I47" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="J47" s="3" t="inlineStr">
@@ -2959,9 +2959,9 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="F48" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
+      <c r="F48" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="G48" s="4" t="inlineStr">
@@ -2969,9 +2969,9 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="H48" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
+      <c r="H48" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="I48" s="4" t="inlineStr">
@@ -3001,9 +3001,9 @@
           <t>Bebas</t>
         </is>
       </c>
-      <c r="D49" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
+      <c r="D49" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="E49" s="4" t="inlineStr">
@@ -3011,14 +3011,14 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="F49" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="G49" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="G49" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="H49" s="4" t="inlineStr">
@@ -3026,9 +3026,9 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="I49" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
+      <c r="I49" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="J49" s="4" t="inlineStr">
@@ -3058,19 +3058,19 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="E50" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="F50" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="G50" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
+      <c r="E50" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="F50" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="G50" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="H50" s="4" t="inlineStr">
@@ -3078,9 +3078,9 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="I50" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
+      <c r="I50" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="J50" s="4" t="inlineStr">
@@ -3105,19 +3105,19 @@
           <t>Bebas</t>
         </is>
       </c>
-      <c r="D51" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="E51" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="F51" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="E51" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="F51" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="G51" s="4" t="inlineStr">
@@ -3130,9 +3130,9 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="I51" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
+      <c r="I51" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="J51" s="4" t="inlineStr">
@@ -3162,9 +3162,9 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="E52" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
+      <c r="E52" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="F52" s="4" t="inlineStr">
@@ -3182,9 +3182,9 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="I52" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
+      <c r="I52" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="J52" s="3" t="inlineStr">
@@ -3219,14 +3219,14 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="F53" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="G53" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
+      <c r="F53" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="G53" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="H53" s="4" t="inlineStr">
@@ -3266,9 +3266,9 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="E54" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="F54" s="4" t="inlineStr">
@@ -3276,14 +3276,14 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="G54" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="H54" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
+      <c r="G54" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="H54" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="I54" s="4" t="inlineStr">
@@ -3291,9 +3291,9 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="J54" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
+      <c r="J54" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
         </is>
       </c>
     </row>
@@ -3318,9 +3318,9 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="E55" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="F55" s="4" t="inlineStr">
@@ -3328,19 +3328,19 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="G55" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="H55" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="I55" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
+      <c r="G55" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="H55" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="I55" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="J55" s="4" t="inlineStr">
@@ -3365,14 +3365,14 @@
           <t>Bebas</t>
         </is>
       </c>
-      <c r="D56" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="E56" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
+        </is>
+      </c>
+      <c r="E56" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="F56" s="4" t="inlineStr">
@@ -3380,9 +3380,9 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="G56" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
+      <c r="G56" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
         </is>
       </c>
       <c r="H56" s="4" t="inlineStr">
@@ -3395,9 +3395,9 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="J56" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
+      <c r="J56" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
         </is>
       </c>
     </row>
@@ -3422,14 +3422,14 @@
           <t>PIKET</t>
         </is>
       </c>
-      <c r="E57" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="F57" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
+      <c r="E57" s="4" t="inlineStr">
+        <is>
+          <t>PIKET</t>
+        </is>
+      </c>
+      <c r="F57" s="3" t="inlineStr">
+        <is>
+          <t>LIBUR</t>
         </is>
       </c>
       <c r="G57" s="4" t="inlineStr">
@@ -3456,64 +3456,64 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>111111111111</t>
+          <t>LS0000243900</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>RusdiEneri</t>
+          <t>Koor QC GSK08_1</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>JUMAT</t>
-        </is>
-      </c>
-      <c r="D58" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="E58" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="F58" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="G58" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
-        </is>
-      </c>
-      <c r="H58" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="I58" s="3" t="inlineStr">
-        <is>
-          <t>LIBUR</t>
-        </is>
-      </c>
-      <c r="J58" s="4" t="inlineStr">
-        <is>
-          <t>PIKET</t>
+          <t>SETIAP HARI</t>
+        </is>
+      </c>
+      <c r="D58" s="5" t="inlineStr">
+        <is>
+          <t>PIKET (LOCKED)</t>
+        </is>
+      </c>
+      <c r="E58" s="5" t="inlineStr">
+        <is>
+          <t>PIKET (LOCKED)</t>
+        </is>
+      </c>
+      <c r="F58" s="5" t="inlineStr">
+        <is>
+          <t>PIKET (LOCKED)</t>
+        </is>
+      </c>
+      <c r="G58" s="5" t="inlineStr">
+        <is>
+          <t>PIKET (LOCKED)</t>
+        </is>
+      </c>
+      <c r="H58" s="5" t="inlineStr">
+        <is>
+          <t>PIKET (LOCKED)</t>
+        </is>
+      </c>
+      <c r="I58" s="5" t="inlineStr">
+        <is>
+          <t>PIKET (LOCKED)</t>
+        </is>
+      </c>
+      <c r="J58" s="5" t="inlineStr">
+        <is>
+          <t>PIKET (LOCKED)</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>LS0000243900</t>
+          <t>LS0000011996</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>Koor QC GSK08_1</t>
+          <t>Qc Monitoring</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
@@ -3552,58 +3552,6 @@
         </is>
       </c>
       <c r="J59" s="5" t="inlineStr">
-        <is>
-          <t>PIKET (LOCKED)</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="2" t="inlineStr">
-        <is>
-          <t>LS0000011996</t>
-        </is>
-      </c>
-      <c r="B60" s="2" t="inlineStr">
-        <is>
-          <t>Qc Monitoring</t>
-        </is>
-      </c>
-      <c r="C60" s="2" t="inlineStr">
-        <is>
-          <t>SETIAP HARI</t>
-        </is>
-      </c>
-      <c r="D60" s="5" t="inlineStr">
-        <is>
-          <t>PIKET (LOCKED)</t>
-        </is>
-      </c>
-      <c r="E60" s="5" t="inlineStr">
-        <is>
-          <t>PIKET (LOCKED)</t>
-        </is>
-      </c>
-      <c r="F60" s="5" t="inlineStr">
-        <is>
-          <t>PIKET (LOCKED)</t>
-        </is>
-      </c>
-      <c r="G60" s="5" t="inlineStr">
-        <is>
-          <t>PIKET (LOCKED)</t>
-        </is>
-      </c>
-      <c r="H60" s="5" t="inlineStr">
-        <is>
-          <t>PIKET (LOCKED)</t>
-        </is>
-      </c>
-      <c r="I60" s="5" t="inlineStr">
-        <is>
-          <t>PIKET (LOCKED)</t>
-        </is>
-      </c>
-      <c r="J60" s="5" t="inlineStr">
         <is>
           <t>PIKET (LOCKED)</t>
         </is>

</xml_diff>